<commit_message>
Three-core requirements spec: sections 4 and 5 cut to one line an item (operating conditions f.sw / f.r / A_e / material, insulation six rows), the resonant-frequency line says the winding current is a half-sine at f.r below resonance and conductors are sized to it; safety rows sized to the wrapped Between column
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Transformer Spec" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F52"/>
+  <dimension ref="B2:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.2" customWidth="1" min="1" max="1"/>
@@ -778,7 +778,7 @@
     <row r="20" ht="38" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Conductors: NP1 Litz, copper ≥ 3.0 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r, copper at 100 °C.</t>
+          <t>Conductors: NP1 Litz, copper ≥ 3.0 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 193 kHz, copper at 100 °C.</t>
         </is>
       </c>
     </row>
@@ -965,11 +965,11 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>at full load; start-up begins at 525 kHz</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
+          <t>full load; start-up 525 kHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="39" customHeight="1">
       <c r="B35" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -987,11 +987,11 @@
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>C.r 75 nF with the three item-2 inductances in series (9.1 µH)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="65" customHeight="1">
+          <t>the winding current is a half-sine at f.r below resonance — conductors are sized to it (C.r 75 nF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="39" customHeight="1">
       <c r="B36" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -1009,11 +1009,11 @@
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>holds the peak flux density at or below 75 mT at f.r with 2 T: B.pk = V.o / (4 · f.r · N.s · Ae).   Ae of the whole flux path — in a flat core the yoke, not the centre leg, usually sets it; two cores in one coil former count together.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="39" customHeight="1">
+          <t>B.pk ≤ 75 mT at f.r with 2 T.   Ae of the flux path: yoke-limited in a flat core; two cores in one former add.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
       <c r="B37" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -1029,73 +1029,115 @@
           <t>MnZn power ferrite, N97 / PC95 / 3C95 class</t>
         </is>
       </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>loss minimum near 100 °C.   The loss budget allows about 1.3 W in the core and 1.0 W in the windings of each transformer at full load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Any core, coil former and winding arrangement meeting sections 2 to 5 is acceptable once the first samples are approved; report the open and leakage inductances, both halves, with the samples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="19" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>5.    SAFETY  INSULATION</t>
         </is>
       </c>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-    </row>
-    <row r="42" ht="14" customHeight="1">
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Household AV (TV) for the US, EU, Japan, Korea and China: IEC 62368-1 as adopted there, GB 4943.1-2022 in China (5000 m).</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="9" t="inlineStr">
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+    </row>
+    <row r="40" ht="14" customHeight="1">
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>IEC 62368-1 (household AV), GB 4943.1-2022 for China; 5000 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C41" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D41" s="9" t="inlineStr">
         <is>
           <t>Between</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="44" customHeight="1">
+    <row r="42" ht="44" customHeight="1">
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Insulation grade</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>primary  |  secondary</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>REINFORCED</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>Primary = NP1, NAUX; secondary = NS2, NS3 and the CORE.   PD 2, OVC II, material group IIIb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="31" customHeight="1">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>Creepage</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>primary  |  secondary</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>≥ 6.4 mm</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>where the triple insulation ends (pins, stripped ends) to the secondary and the core</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="31" customHeight="1">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Insulation grade</t>
+          <t>Clearance</t>
         </is>
       </c>
       <c r="D44" s="18" t="inlineStr">
@@ -1105,24 +1147,24 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>REINFORCED</t>
+          <t>≥ 4.5 mm</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>Primary = NP1, NAUX; secondary = NS2, NS3 and the CORE. Pollution degree 2, overvoltage category II, material group IIIb, 5000 m.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="57" customHeight="1">
+          <t>at 5000 m (3.0 mm × 1.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="44" customHeight="1">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Creepage</t>
+          <t>NP1, NAUX wire</t>
         </is>
       </c>
       <c r="D45" s="18" t="inlineStr">
@@ -1132,24 +1174,24 @@
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>≥ 6.4 mm</t>
+          <t>TIW, reinforced</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Wherever the triple insulation ends: primary pins and stripped wire ends to the core and to secondary leads and pins (320 V rms row, reinforced = 2 × basic).</t>
+          <t>triple-insulated (NP1: TIW-Litz), approved to IEC 62368-1 up to 525 kHz; one wire pin to pin</t>
         </is>
       </c>
     </row>
     <row r="46" ht="31" customHeight="1">
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Clearance</t>
+          <t>Solid insulation</t>
         </is>
       </c>
       <c r="D46" s="18" t="inlineStr">
@@ -1159,157 +1201,75 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>≥ 4.5 mm</t>
+          <t>DTI ≥ 0.4 mm  or  ≥ 2 tape layers</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>3.0 mm at 2000 m × 1.48 for 5000 m, rounded up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="44" customHeight="1">
+          <t>where tape or sleeving carries it</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="31" customHeight="1">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>NP1 wire</t>
+          <t>Electric strength</t>
         </is>
       </c>
       <c r="D47" s="18" t="inlineStr">
         <is>
-          <t>NP1  |  secondary</t>
+          <t>primary  |  secondary</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>TIW-Litz, reinforced</t>
+          <t>3000 V ac 60 s  (4242 V dc)</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Triple-insulated Litz approved as reinforced insulation to IEC 62368-1, one wire from pin to pin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="70" customHeight="1">
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>NAUX wire</t>
-        </is>
-      </c>
-      <c r="D48" s="18" t="inlineStr">
-        <is>
-          <t>NAUX  |  secondary</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>TIW, reinforced</t>
-        </is>
-      </c>
-      <c r="F48" s="11" t="inlineStr">
-        <is>
-          <t>Triple-insulated wire approved as reinforced insulation to IEC 62368-1; leads stay insulated up to the primary pins. Its approved frequency must cover the start-up frequency, 525 kHz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="57" customHeight="1">
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>Solid insulation</t>
-        </is>
-      </c>
-      <c r="D49" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>DTI ≥ 0.4 mm  or  ≥ 2 tape layers</t>
-        </is>
-      </c>
-      <c r="F49" s="11" t="inlineStr">
-        <is>
-          <t>Where tape or sleeving carries it: each tape layer passes the reinforced test. Sleeve primary leads that leave the triple insulation near the core.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="57" customHeight="1">
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>Electric strength</t>
-        </is>
-      </c>
-      <c r="D50" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>3000 V ac 60 s  (4242 V dc)</t>
-        </is>
-      </c>
-      <c r="F50" s="11" t="inlineStr">
-        <is>
-          <t>NP1 + NAUX joined against NS2 + NS3 + core joined. Type test, no breakdown. Routine test voltage and time as agreed with the certifier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>The working voltage behind item 2 is an estimate from the design (187 V rms, 373 V peak at 264 Vac); the certifying body measures it.</t>
+          <t>NP1 + NAUX against NS2 + NS3 + core; type test, no breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="14" customHeight="1">
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Working voltage: design estimate 187 V rms / 373 V peak at 264 Vac; the certifying body measures it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="24">
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="C35:D35"/>
-    <mergeCell ref="B52:F52"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B42:F42"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="C36:D36"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B49:F49"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="C37:D37"/>
-    <mergeCell ref="B41:F41"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Three-core requirements spec: above-resonance operation is not rare - the line-cycle sweep puts the line peaks above f.r from 105 Vac FB and 209 Vac HB (110 Vac 20 % of the time / 39 % of the energy, 230 Vac 27 / 51 %, 264 Vac 42 / 73 %, load-independent), so the resonant-frequency line says sine at f.sw above resonance and the conductor note gives the skin depth at 307 kHz as well; notes corrected
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -778,7 +778,7 @@
     <row r="20" ht="38" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Conductors: NP1 Litz, copper ≥ 3.0 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 193 kHz, copper at 100 °C.</t>
+          <t>Conductors: NP1 Litz, copper ≥ 3.0 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 193 kHz and 0.14 mm at 307 kHz, copper at 100 °C.</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="39" customHeight="1">
+    <row r="35" ht="52" customHeight="1">
       <c r="B35" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -987,7 +987,7 @@
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>the winding current is a half-sine at f.r below resonance — conductors are sized to it (C.r 75 nF)</t>
+          <t>winding current: half-sine at f.r below resonance, sine at f.sw above it (around the line peaks) — conductors sized for the top of the range (C.r 75 nF)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Three-core third option moved to round numbers: C.r 70.5 nF (TDK C4532C0G2J473 C0G, 2 series x 3 parallel), L.r 10 uH, L.m 15 uH (set 10 / 25 uH, a unit 3.33 / 8.33 uH), R.T 7.68 k so f.Min sits 8 % above f.o again; f.r 189.6 kHz, 71/75 at the nominal, at every +-10 % inductance corner and at L.r 8 / 11 uH re-centred; L.open 24 would leave k.floor 1.035, 27 k.ZVS 1.32, 30 fails; variant sheet and requirements spec rebuilt, canonical sheet unchanged
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>11.0 A   /   18.3 A</t>
+          <t>10.9 A   /   18.2 A</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>9.3 A   /   32.0 A</t>
+          <t>9.2 A   /   31.2 A</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>9.3 A   /   32.0 A</t>
+          <t>9.2 A   /   31.2 A</t>
         </is>
       </c>
     </row>
@@ -757,14 +757,14 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>174 mA dc load (VCC)</t>
+          <t>175 mA dc load (VCC)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.   One conductor per pin; a secondary pin carries its whole winding current (9.3 A rms): confirm the pin current rating, or bring the secondary ends straight out.</t>
+          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.   One conductor per pin; a secondary pin carries its whole winding current (9.2 A rms): confirm the pin current rating, or bring the secondary ends straight out.</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
     <row r="20" ht="38" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Conductors: NP1 Litz, copper ≥ 3.0 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 193 kHz and 0.14 mm at 307 kHz, copper at 100 °C.</t>
+          <t>Conductors: NP1 Litz, copper ≥ 2.9 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 190 kHz and 0.14 mm at 292 kHz, copper at 100 °C.</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>8.03 µH    ±10 %</t>
+          <t>8.33 µH    ±10 %</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>3.03 µH    ±10 %</t>
+          <t>3.33 µH    ±10 %</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -918,14 +918,14 @@
     <row r="29" ht="26" customHeight="1">
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Both measured at 1 – 2 of ONE transformer.   Three in series give the set 24.1 µH open and 9.1 µH leakage, and the ratio 7.5 : 1.</t>
+          <t>Both measured at 1 – 2 of ONE transformer.   Three in series give the set 25.0 µH open and 10.0 µH leakage, and the ratio 7.5 : 1.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="50" customHeight="1">
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Item 2 is the resonant inductor: C.r 75 nF with the three in series gives f.r 193 kHz.   If the construction cannot reach it, quote the value it reaches BEFORE samples: 2.67 to 3.67 µH per transformer is taken by re-selecting C.r and the oscillator setting, the ±10 % then applying around the quoted value; below that the difference goes into an external inductor.</t>
+          <t>Item 2 is the resonant inductor: C.r 70.5 nF with the three in series gives f.r 190 kHz.   If the construction cannot reach it, quote the value it reaches BEFORE samples: 2.67 to 3.67 µH per transformer is taken by re-selecting C.r and the oscillator setting, the ±10 % then applying around the quoted value; below that the difference goes into an external inductor.</t>
         </is>
       </c>
     </row>
@@ -960,12 +960,12 @@
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>127  to  307 kHz</t>
+          <t>130  to  292 kHz</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>full load; start-up 525 kHz</t>
+          <t>full load; start-up 527 kHz</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>f.r  193 kHz</t>
+          <t>f.r  190 kHz</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>winding current: half-sine at f.r below resonance, sine at f.sw above it (around the line peaks) — conductors sized for the top of the range (C.r 75 nF)</t>
+          <t>winding current: half-sine at f.r below resonance, sine at f.sw above it (around the line peaks) — conductors sized for the top of the range (C.r 70.5 nF)</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>triple-insulated (NP1: TIW-Litz), approved to IEC 62368-1 up to 525 kHz; one wire pin to pin</t>
+          <t>triple-insulated (NP1: TIW-Litz), approved to IEC 62368-1 up to 527 kHz; one wire pin to pin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Three-core requirements spec: no safety-insulation section (the customer's safety engineering writes it), operating conditions reduced to the frequency the windings see and the core area, the resonant-frequency and core-material lines dropped; one-transformer spec unchanged
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Transformer Spec" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -177,13 +177,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F49"/>
+  <dimension ref="B2:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.2" customWidth="1" min="1" max="1"/>
@@ -611,7 +605,7 @@
     <row r="9" ht="28" customHeight="1">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>•   Flat (low-profile) construction as the production part 26OP-LM83W.   Core, coil former, wire and winding arrangement are the supplier’s choice within sections 2 to 5; the overall height is agreed with the set mechanical design before the first samples.</t>
+          <t>•   Flat (low-profile) construction as the production part 26OP-LM83W.   Core, coil former, wire and winding arrangement are the supplier’s choice within sections 2 to 4; the overall height is agreed with the set mechanical design before the first samples.</t>
         </is>
       </c>
     </row>
@@ -778,7 +772,7 @@
     <row r="20" ht="38" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Conductors: NP1 Litz, copper ≥ 2.9 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at f.r 190 kHz and 0.14 mm at 292 kHz, copper at 100 °C.</t>
+          <t>Conductors: NP1 Litz, copper ≥ 2.9 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at 190 kHz and 0.14 mm at 292 kHz, copper at 100 °C.</t>
         </is>
       </c>
     </row>
@@ -925,7 +919,7 @@
     <row r="30" ht="50" customHeight="1">
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Item 2 is the resonant inductor: C.r 70.5 nF with the three in series gives f.r 190 kHz.   If the construction cannot reach it, quote the value it reaches BEFORE samples: 2.67 to 3.67 µH per transformer is taken by re-selecting C.r and the oscillator setting, the ±10 % then applying around the quoted value; below that the difference goes into an external inductor.</t>
+          <t>Item 2 is the converter’s resonant inductor (190 kHz with C.r 70.5 nF).   If the construction cannot reach it, quote the value it reaches BEFORE samples: 2.67 to 3.67 µH per transformer is taken by re-selecting C.r and the oscillator setting, the ±10 % then applying around the quoted value; below that the difference goes into an external inductor.</t>
         </is>
       </c>
     </row>
@@ -947,7 +941,7 @@
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
     </row>
-    <row r="34" ht="16" customHeight="1">
+    <row r="34" ht="26" customHeight="1">
       <c r="B34" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -955,7 +949,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Switching frequency</t>
+          <t>Operating frequency</t>
         </is>
       </c>
       <c r="E34" s="16" t="inlineStr">
@@ -963,13 +957,13 @@
           <t>130  to  292 kHz</t>
         </is>
       </c>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t>full load; start-up 527 kHz</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="52" customHeight="1">
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>of the winding current and voltage at full load; start-up 527 kHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="39" customHeight="1">
       <c r="B35" s="15" t="inlineStr">
         <is>
           <t>•</t>
@@ -977,275 +971,22 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Resonant frequency</t>
-        </is>
-      </c>
-      <c r="E35" s="17" t="inlineStr">
-        <is>
-          <t>f.r  190 kHz</t>
+          <t>Core effective area</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Ae  ≥  220 mm²</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>winding current: half-sine at f.r below resonance, sine at f.sw above it (around the line peaks) — conductors sized for the top of the range (C.r 70.5 nF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="39" customHeight="1">
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Core effective area</t>
-        </is>
-      </c>
-      <c r="E36" s="17" t="inlineStr">
-        <is>
-          <t>Ae  ≥  220 mm²</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>B.pk ≤ 75 mT at f.r with 2 T.   Ae of the flux path: yoke-limited in a flat core; two cores in one former add.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Core material</t>
-        </is>
-      </c>
-      <c r="E37" s="17" t="inlineStr">
-        <is>
-          <t>MnZn power ferrite, N97 / PC95 / 3C95 class</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="19" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>5.    SAFETY  INSULATION</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-    </row>
-    <row r="40" ht="14" customHeight="1">
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>IEC 62368-1 (household AV), GB 4943.1-2022 for China; 5000 m.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Between</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>Requirement</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="44" customHeight="1">
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>Insulation grade</t>
-        </is>
-      </c>
-      <c r="D42" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>REINFORCED</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="inlineStr">
-        <is>
-          <t>Primary = NP1, NAUX; secondary = NS2, NS3 and the CORE.   PD 2, OVC II, material group IIIb.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="31" customHeight="1">
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>Creepage</t>
-        </is>
-      </c>
-      <c r="D43" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>≥ 6.4 mm</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="inlineStr">
-        <is>
-          <t>where the triple insulation ends (pins, stripped ends) to the secondary and the core</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="31" customHeight="1">
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>Clearance</t>
-        </is>
-      </c>
-      <c r="D44" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>≥ 4.5 mm</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
-        <is>
-          <t>at 5000 m (3.0 mm × 1.48)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="44" customHeight="1">
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>NP1, NAUX wire</t>
-        </is>
-      </c>
-      <c r="D45" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>TIW, reinforced</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="inlineStr">
-        <is>
-          <t>triple-insulated (NP1: TIW-Litz), approved to IEC 62368-1 up to 527 kHz; one wire pin to pin</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="31" customHeight="1">
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>Solid insulation</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>DTI ≥ 0.4 mm  or  ≥ 2 tape layers</t>
-        </is>
-      </c>
-      <c r="F46" s="11" t="inlineStr">
-        <is>
-          <t>where tape or sleeving carries it</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="31" customHeight="1">
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>Electric strength</t>
-        </is>
-      </c>
-      <c r="D47" s="18" t="inlineStr">
-        <is>
-          <t>primary  |  secondary</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>3000 V ac 60 s  (4242 V dc)</t>
-        </is>
-      </c>
-      <c r="F47" s="11" t="inlineStr">
-        <is>
-          <t>NP1 + NAUX against NS2 + NS3 + core; type test, no breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="14" customHeight="1">
-      <c r="B49" s="14" t="inlineStr">
-        <is>
-          <t>Working voltage: design estimate 187 V rms / 373 V peak at 264 Vac; the certifying body measures it.</t>
+          <t>B.pk ≤ 75 mT with 2 T at 190 kHz.   Ae of the flux path: yoke-limited in a flat core; two cores in one former add.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="19">
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B3:F3"/>
@@ -1253,23 +994,18 @@
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B39:F39"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B19:F19"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="B40:F40"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B49:F49"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B33:F33"/>
-    <mergeCell ref="C37:D37"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Three-core requirements spec written purely from the transformer's side: no converter, set-connection or resonant-tank statements, turns 5 : 2 : 2 : 1 in the title, construction / winding / electrical / operating conditions only; a Korean edition from the same builder with --kr (string table, Malgun Gothic); one-transformer spec unchanged
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Transformer Spec" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Transformer Spec'!$A$1:$G$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,12 +47,6 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -133,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -147,15 +141,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -164,19 +152,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -544,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F35"/>
+  <dimension ref="B2:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.2" customWidth="1" min="1" max="1"/>
@@ -566,7 +557,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>L6790A single-stage PF LLC converter      25 V / 26.3 A output      —      turns ratio 7.5 : 1</t>
+          <t>Turns   NP1 : NS2 : NS3 : NAUX   =   5 : 2 : 2 : 1</t>
         </is>
       </c>
     </row>
@@ -580,7 +571,7 @@
     <row r="6" ht="19" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>1.    CONFIGURATION</t>
+          <t>1.    CONSTRUCTION</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -588,424 +579,400 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>•   Three identical transformers per set — primaries in series, secondaries in parallel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>•   EVERY VALUE BELOW IS PER TRANSFORMER.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>•   Flat (low-profile) construction as the production part 26OP-LM83W.   Core, coil former, wire and winding arrangement are the supplier’s choice within sections 2 to 4; the overall height is agreed with the set mechanical design before the first samples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="19" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+          <t>•   Flat (low-profile) construction as the production part 26OP-LM83W.   Core, coil former, wire and winding arrangement are the supplier’s choice within sections 2 to 4; the overall height is agreed before the first samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>2.    WINDING</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Winding</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Turns</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Winding current           rms   /   peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>NP1     Primary</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>5 T</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>10.9 A   /   18.2 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Winding</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+          <t>NS2     Secondary A</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>3 – 5</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>2 T</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>9.2 A   /   31.2 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>NS3     Secondary B</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>2 T</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>9.2 A   /   31.2 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>NAUX   Auxiliary</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>a – b</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>1 T</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>175 mA dc</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.   One conductor per pin; a secondary pin carries its whole winding current (9.2 A rms): confirm the pin current rating, or bring the secondary ends straight out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Terminal numbers follow the production part 26OP-LM83W (approval sheet, KH Feelux): primary 1 – 2, secondaries 3 – 5 and 4 – 6, auxiliary a – b.   Pin layout is the supplier’s choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Conductors: NP1 Litz, copper ≥ 2.9 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at 190 kHz and 0.14 mm at 292 kHz, copper at 100 °C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>NAUX: 1 T on every transformer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="19" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>3.    ELECTRICAL  REQUIREMENTS</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Measured with an LCR meter at 100 kHz / 1 V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Turns</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Winding current           rms   /   peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="31" customHeight="1">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>NP1     Primary</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>INDUCTANCE</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>1 – 2</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>5 T</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>10.9 A   /   18.2 A</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="10" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>8.33 µH    ±10 %</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>All other windings OPEN.   L.mag + L.leak, not L.mag alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>NS2     Secondary A</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>3 – 5</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>2 T</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>9.2 A   /   31.2 A</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>LEAKAGE INDUCTANCE</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>3.33 µH    ±10 %</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>EACH HALF: NS2 short alone, then NS3 short alone; the other half and NAUX open.   Both must pass.   A target, not a maximum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>NS3     Secondary B</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>2 T</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>9.2 A   /   31.2 A</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>NAUX   Auxiliary (VCC, ZCD)</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>a – b</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>1 T</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>175 mA dc load (VCC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="38" customHeight="1">
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Centre tap is made on the PCB by joining pins 4 and 5 — do NOT join them inside the transformer.   One conductor per pin; a secondary pin carries its whole winding current (9.2 A rms): confirm the pin current rating, or bring the secondary ends straight out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>Terminal numbers follow the production part 26OP-LM83W (approval sheet, KH Feelux): primary 1 – 2, secondaries 3 – 5 and 4 – 6, auxiliary a – b.   Pin layout is the supplier’s choice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="38" customHeight="1">
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>Conductors: NP1 Litz, copper ≥ 2.9 mm², strands ≤ 0.10 mm.   NS2 and NS3 each: Litz (strands ≤ 0.10 mm) or copper foil ≤ 0.20 mm thick, copper ≥ 2.5 mm².   From 3.75 A/mm² at the rms currents above; skin depth 0.17 mm at 190 kHz and 0.14 mm at 292 kHz, copper at 100 °C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="14" customHeight="1">
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>NAUX: 1 T on EVERY transformer; the set series-connects two of them (2 T in all), the other one stays open.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="19" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>3.    ELECTRICAL  REQUIREMENTS</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="14" customHeight="1">
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>Measured with an LCR meter at 100 kHz / 1 V.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>Requirement</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="31" customHeight="1">
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>INDUCTANCE</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>D.C OVERLAP</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>1 – 2</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>8.33 µH    ±10 %</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>All other windings OPEN.   L.mag + L.leak, not L.mag alone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="57" customHeight="1">
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>LEAKAGE INDUCTANCE</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>1 – 2</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>3.33 µH    ±10 %</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>EACH HALF: NS2 short alone, then NS3 short alone; the other half and NAUX open.   Both must pass.   Resonant inductor — a target, not a maximum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>D.C OVERLAP</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>1 – 2</t>
-        </is>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>≥ 90 % of initial inductance</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Test current 17 A, normal temperature</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Both measured at 1 – 2 of ONE transformer.   Three in series give the set 25.0 µH open and 10.0 µH leakage, and the ratio 7.5 : 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="50" customHeight="1">
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Item 2 is the converter’s resonant inductor (190 kHz with C.r 70.5 nF).   If the construction cannot reach it, quote the value it reaches BEFORE samples: 2.67 to 3.67 µH per transformer is taken by re-selecting C.r and the oscillator setting, the ±10 % then applying around the quoted value; below that the difference goes into an external inductor.</t>
-        </is>
-      </c>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Item 2 is a target, not a maximum: if the construction cannot reach it, state the value it reaches BEFORE samples — 2.67 to 3.67 µH is acceptable, the ±10 % then applying around the stated value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>With NS2 and NS3 both shorted the reading is lower: record it, do not hold it to item 2.   The auxiliary is NOT shorted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>4.    OPERATING  CONDITIONS</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>With NS2 and NS3 both shorted the reading is lower: record it, do not hold it to item 2.   The auxiliary is NOT shorted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>4.    OPERATING  CONDITIONS</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="B34" s="15" t="inlineStr">
-        <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>Operating frequency</t>
-        </is>
-      </c>
-      <c r="E34" s="16" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Winding frequency</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>130  to  292 kHz</t>
         </is>
       </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>of the winding current and voltage at full load; start-up 527 kHz</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="39" customHeight="1">
-      <c r="B35" s="15" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>of the winding current and voltage at full load; up to 527 kHz briefly at start-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="39" customHeight="1">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>Core effective area</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Ae  ≥  220 mm²</t>
         </is>
       </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>B.pk ≤ 75 mT with 2 T at 190 kHz.   Ae of the flux path: yoke-limited in a flat core; two cores in one former add.</t>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>keeps B.pk ≤ 75 mT with 2 T at 190 kHz.   Ae of the whole flux path: yoke-limited in a flat core; two cores in one former add.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C34:D34"/>
+  <mergeCells count="16">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B30:F30"/>
     <mergeCell ref="B7:F7"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B18:F18"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B29:F29"/>
     <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="B17:F17"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B27:F27"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
LG transformer core: the outline drawing measured at 600 dpi with its own 143.9 mm dimension shows a 66.9 mm core region (2 x 33.5) split exactly in the middle in both views, with one fixing-tape band centred on each half - two EE6405 pairs (four halves) butted along the depth; the QC chart in that spec belongs to another model. Requirements spec wording: "two core sets (pairs) side by side" instead of "two cores"
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3.xlsx
@@ -933,7 +933,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="39" customHeight="1">
+    <row r="32" ht="52" customHeight="1">
       <c r="B32" s="13" t="inlineStr">
         <is>
           <t>•</t>
@@ -951,7 +951,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>keeps B.pk ≤ 75 mT with 2 T at 190 kHz.   Ae of the whole flux path: yoke-limited in a flat core; two cores in one former add.</t>
+          <t>keeps B.pk ≤ 75 mT with 2 T at 190 kHz.   Ae of the whole flux path: yoke-limited in a flat core; two core sets (pairs) placed side by side in one former add.</t>
         </is>
       </c>
     </row>

</xml_diff>